<commit_message>
fixing some errors, adding examples
</commit_message>
<xml_diff>
--- a/StructureDefinition-ophthalmic-diagnostic-report.xlsx
+++ b/StructureDefinition-ophthalmic-diagnostic-report.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-18T20:04:06+00:00</t>
+    <t>2026-08-19T17:13:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -4363,7 +4363,7 @@
         <v>79</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>92</v>

</xml_diff>